<commit_message>
chore(demo3): update Excel scene Tip values to new type system
Scene 4: static_orbit → cameras
Scene 5: pointerlock (FPS) → walkthru
Scenes 0-3: orbit (already correct)

https://claude.ai/code/session_01NbLjFLHf9cNBKyb3QMv6fy
</commit_message>
<xml_diff>
--- a/demo3/demo3-input_4.xlsx
+++ b/demo3/demo3-input_4.xlsx
@@ -25334,7 +25334,7 @@
       </c>
       <c r="B498" s="19" t="inlineStr">
         <is>
-          <t>static_orbit</t>
+          <t>cameras</t>
         </is>
       </c>
       <c r="C498" s="19" t="n"/>
@@ -30691,7 +30691,7 @@
       </c>
       <c r="B611" s="19" t="inlineStr">
         <is>
-          <t>pointerlock  (FPS)</t>
+          <t>walkthru</t>
         </is>
       </c>
       <c r="C611" s="19" t="n"/>

</xml_diff>

<commit_message>
feat: integrate FURNITURE_EDIT and FURNITURE_VIEW toggles into cameras mode (Prompt 4/7)
- Extract _switchToPlanView/_switchToPerspView helpers from enterClipMode/exitClipMode
- Add enterFurnitureEdit: plan view + FurniturePanel + FurnitureEditor active + selection info panel
- Add enterFurnitureView: plan view + placed items list from cache
- Add exitFurnitureMode: deactivate editor, hide panels, unsuspend hotspots
- Canvas click selects furniture items, drag-drop spawns from panel
- Keyboard shortcuts: R=rotate, T=translate, Delete=remove
- Excel: add rows 8 (Mobilya Editörü/FURNITURE_EDIT) and 9 (Mobilya Görünüm/FURNITURE_VIEW)

https://claude.ai/code/session_013hU48LyzRTRPw4KksUQhoP
</commit_message>
<xml_diff>
--- a/demo3/demo3-input_4.xlsx
+++ b/demo3/demo3-input_4.xlsx
@@ -26671,29 +26671,27 @@
       <c r="O525" s="21" t="n"/>
     </row>
     <row r="526">
-      <c r="A526" s="21" t="inlineStr">
-        <is>
-          <t>slot08</t>
-        </is>
+      <c r="A526" s="21" t="n">
+        <v>8</v>
       </c>
       <c r="B526" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Mobilya Editörü</t>
         </is>
       </c>
       <c r="C526" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>furnEdit</t>
         </is>
       </c>
       <c r="D526" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>FURNITURE_EDIT</t>
         </is>
       </c>
       <c r="E526" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-3</t>
         </is>
       </c>
       <c r="F526" s="21" t="n"/>
@@ -26708,29 +26706,27 @@
       <c r="O526" s="21" t="n"/>
     </row>
     <row r="527">
-      <c r="A527" s="21" t="inlineStr">
-        <is>
-          <t>slot09</t>
-        </is>
+      <c r="A527" s="21" t="n">
+        <v>9</v>
       </c>
       <c r="B527" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Mobilya Görünüm</t>
         </is>
       </c>
       <c r="C527" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>furnView</t>
         </is>
       </c>
       <c r="D527" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>FURNITURE_VIEW</t>
         </is>
       </c>
       <c r="E527" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-3-view</t>
         </is>
       </c>
       <c r="F527" s="21" t="n"/>

</xml_diff>

<commit_message>
fix: clip plane formula, action matching, Excel camera config
1. CLIP_MODE action matching: === 'CLIP_MODE' → startsWith('CLIP_MODE')
   so plan view actually works again (was broken by ·40 suffix)
2. Clip plane formula INVERTED: was maxY - pct*h (backwards), now
   minY + pct*h — low % = floor plan only, high % = show more building
3. BBox: scene.updateMatrixWorld(true) before compute, explicit skip
   for TransformControls gizmo/plane meshes via parent-walk
4. Excel: clip height moved to camera config "Clip Height %" = 40
   (separate field in 1·KAMERA section, not encoded in action string)
5. Reverted CLIP_MODE·40 back to plain CLIP_MODE in toggle buttons

https://claude.ai/code/session_013hU48LyzRTRPw4KksUQhoP
</commit_message>
<xml_diff>
--- a/demo3/demo3-input_4.xlsx
+++ b/demo3/demo3-input_4.xlsx
@@ -25369,8 +25369,14 @@
         </is>
       </c>
       <c r="L498" s="19" t="n"/>
-      <c r="M498" s="19" t="n"/>
-      <c r="N498" s="19" t="n"/>
+      <c r="M498" s="19" t="inlineStr">
+        <is>
+          <t>Clip Height %</t>
+        </is>
+      </c>
+      <c r="N498" s="19" t="n">
+        <v>40</v>
+      </c>
       <c r="O498" s="19" t="n"/>
     </row>
     <row r="499">

</xml_diff>

<commit_message>
chore: update Excel — Auto-Rotate mouse-break, camera positions, clip config
- Scene 1+2: Auto-Rotate changed from YES to mouse-break
- Scene 4 cameras: updated Pos/LookAt/FOV + nav dot positions for all 6 rooms
- CLIP_MODE action reverted to plain (clip % now in camera config)
- Clip Height % = 40 in camera config section (row 498, col M-N)

https://claude.ai/code/session_013hU48LyzRTRPw4KksUQhoP
</commit_message>
<xml_diff>
--- a/demo3/demo3-input_4.xlsx
+++ b/demo3/demo3-input_4.xlsx
@@ -8734,7 +8734,7 @@
       </c>
       <c r="B158" s="19" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>mouse-break</t>
         </is>
       </c>
       <c r="C158" s="19" t="n"/>
@@ -14273,7 +14273,7 @@
       </c>
       <c r="B272" s="19" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>mouse-break</t>
         </is>
       </c>
       <c r="C272" s="19" t="n"/>
@@ -26447,7 +26447,7 @@
       </c>
       <c r="D519" s="19" t="inlineStr">
         <is>
-          <t>Pos(1, 1.6, 1.6)   → LookAt(1, 1.6, 1.5)   · FOV 80</t>
+          <t>Pos(1.429, 1.607, 1.852)   → LookAt(1.000, 1.600, 1.500)   · FOV 80</t>
         </is>
       </c>
       <c r="E519" s="19" t="inlineStr">
@@ -26455,9 +26455,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F519" s="19" t="n"/>
-      <c r="G519" s="19" t="n"/>
-      <c r="H519" s="19" t="n"/>
+      <c r="F519" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G519" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H519" s="19" t="n">
+        <v>1.6</v>
+      </c>
       <c r="I519" s="19" t="n"/>
       <c r="J519" s="19" t="n"/>
       <c r="K519" s="19" t="n"/>
@@ -26482,7 +26488,7 @@
       </c>
       <c r="D520" s="19" t="inlineStr">
         <is>
-          <t>Pos(-2, 1.6, 3.1)  → LookAt(-2.1, 1.6, 3.2) · FOV 80</t>
+          <t>Pos(-1.136, 1.650, 3.398)   → LookAt(-2.125, 1.600, 3.200)   · FOV 80</t>
         </is>
       </c>
       <c r="E520" s="19" t="inlineStr">
@@ -26490,9 +26496,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F520" s="19" t="n"/>
-      <c r="G520" s="19" t="n"/>
-      <c r="H520" s="19" t="n"/>
+      <c r="F520" s="19" t="n">
+        <v>-1.299</v>
+      </c>
+      <c r="G520" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H520" s="19" t="n">
+        <v>3.478</v>
+      </c>
       <c r="I520" s="19" t="n"/>
       <c r="J520" s="19" t="n"/>
       <c r="K520" s="19" t="n"/>
@@ -26517,7 +26529,7 @@
       </c>
       <c r="D521" s="19" t="inlineStr">
         <is>
-          <t>Pos(-2, 1.6, 0)    → LookAt(-2.1, 1.6, -0.1) · FOV 80</t>
+          <t>Pos(-2.000, 1.600, 0.000)   → LookAt(-2.100, 1.600, -0.100)   · FOV 80</t>
         </is>
       </c>
       <c r="E521" s="19" t="inlineStr">
@@ -26525,9 +26537,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F521" s="19" t="n"/>
-      <c r="G521" s="19" t="n"/>
-      <c r="H521" s="19" t="n"/>
+      <c r="F521" s="19" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G521" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H521" s="19" t="n">
+        <v>0</v>
+      </c>
       <c r="I521" s="19" t="n"/>
       <c r="J521" s="19" t="n"/>
       <c r="K521" s="19" t="n"/>
@@ -26552,7 +26570,7 @@
       </c>
       <c r="D522" s="19" t="inlineStr">
         <is>
-          <t>Pos(-2, 1.6, 2.1)  → LookAt(-2.1, 1.6, 2.2) · FOV 80</t>
+          <t>Pos(-2.000, 1.600, 2.100)   → LookAt(-2.100, 1.600, 2.200)   · FOV 80</t>
         </is>
       </c>
       <c r="E522" s="19" t="inlineStr">
@@ -26560,9 +26578,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F522" s="19" t="n"/>
-      <c r="G522" s="19" t="n"/>
-      <c r="H522" s="19" t="n"/>
+      <c r="F522" s="19" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="G522" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H522" s="19" t="n">
+        <v>2.1</v>
+      </c>
       <c r="I522" s="19" t="n"/>
       <c r="J522" s="19" t="n"/>
       <c r="K522" s="19" t="n"/>
@@ -26587,7 +26611,7 @@
       </c>
       <c r="D523" s="19" t="inlineStr">
         <is>
-          <t>Pos(4.4, 1.6, 0)   → LookAt(4.5, 1.6, -0.1) · FOV 80</t>
+          <t>Pos(5.640, 1.600, 2.139)   → LookAt(4.500, 1.600, -0.100)   · FOV 80</t>
         </is>
       </c>
       <c r="E523" s="19" t="inlineStr">
@@ -26595,9 +26619,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F523" s="19" t="n"/>
-      <c r="G523" s="19" t="n"/>
-      <c r="H523" s="19" t="n"/>
+      <c r="F523" s="19" t="n">
+        <v>5.138</v>
+      </c>
+      <c r="G523" s="19" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="H523" s="19" t="n">
+        <v>2.021</v>
+      </c>
       <c r="I523" s="19" t="n"/>
       <c r="J523" s="19" t="n"/>
       <c r="K523" s="19" t="n"/>
@@ -26622,7 +26652,7 @@
       </c>
       <c r="D524" s="19" t="inlineStr">
         <is>
-          <t>Pos(3.9, 1.6, 3.7) → LookAt(4.0, 1.6, 3.8) · FOV 80</t>
+          <t>Pos(4.930, 1.691, 3.838)   → LookAt(4.000, 1.600, 3.800)   · FOV 80</t>
         </is>
       </c>
       <c r="E524" s="19" t="inlineStr">
@@ -26630,9 +26660,15 @@
           <t>toggle-1</t>
         </is>
       </c>
-      <c r="F524" s="19" t="n"/>
-      <c r="G524" s="19" t="n"/>
-      <c r="H524" s="19" t="n"/>
+      <c r="F524" s="19" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="G524" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H524" s="19" t="n">
+        <v>3.736</v>
+      </c>
       <c r="I524" s="19" t="n"/>
       <c r="J524" s="19" t="n"/>
       <c r="K524" s="19" t="n"/>
@@ -26657,7 +26693,7 @@
       </c>
       <c r="D525" s="21" t="inlineStr">
         <is>
-          <t>CLIP_MODE·40</t>
+          <t>CLIP_MODE</t>
         </is>
       </c>
       <c r="E525" s="21" t="inlineStr">

</xml_diff>

<commit_message>
fix: swap scene 4↔5 numbering, startup bug, shared cache, clear button
1. Excel: Scene 4 = Mobilya Editörü (row 608, SAHNE 4), Scene 5 = İç Mekan
   Kameraları (row 494, SAHNE 5). Loader reads by marker number, not row order.
2. Scene 5: removed FURNITURE_EDIT/VIEW toggles, keeps only camera positions
   + Plan Görünümü (CLIP_MODE)
3. Startup bug: first button action checked — if CLIP_MODE, auto-enter
   plan view instead of broken selectCamera(0) with null position
4. Shared furniture cache: cacheKey = 'vea-furniture-interior' across all
   interior scenes — furniture placed in scene 4 visible in scene 5
5. "Tümünü Temizle" button in furniture edit right panel when nothing
   selected — removes all placed items

https://claude.ai/code/session_013hU48LyzRTRPw4KksUQhoP
</commit_message>
<xml_diff>
--- a/demo3/demo3-input_4.xlsx
+++ b/demo3/demo3-input_4.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S836"/>
+  <dimension ref="A1:O836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -25214,7 +25214,7 @@
     <row r="494">
       <c r="A494" s="7" t="inlineStr">
         <is>
-          <t>▌ SAHNE 4  —  İç Mekan  ·  6 Kamera Pozisyonu  (Statik + Orbit)</t>
+          <t>▌ SAHNE 5  —  İç Mekan  ·  6 Kamera Pozisyonu  (Statik + Orbit)</t>
         </is>
       </c>
       <c r="B494" s="7" t="n"/>
@@ -26713,27 +26713,29 @@
       <c r="O525" s="21" t="n"/>
     </row>
     <row r="526">
-      <c r="A526" s="21" t="n">
-        <v>8</v>
+      <c r="A526" s="21" t="inlineStr">
+        <is>
+          <t>slot08</t>
+        </is>
       </c>
       <c r="B526" s="21" t="inlineStr">
         <is>
-          <t>Mobilya Editörü</t>
+          <t>null</t>
         </is>
       </c>
       <c r="C526" s="21" t="inlineStr">
         <is>
-          <t>furnEdit</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D526" s="21" t="inlineStr">
         <is>
-          <t>FURNITURE_EDIT</t>
+          <t>null</t>
         </is>
       </c>
       <c r="E526" s="21" t="inlineStr">
         <is>
-          <t>toggle-3</t>
+          <t>null</t>
         </is>
       </c>
       <c r="F526" s="21" t="n"/>
@@ -26748,27 +26750,29 @@
       <c r="O526" s="21" t="n"/>
     </row>
     <row r="527">
-      <c r="A527" s="21" t="n">
-        <v>9</v>
+      <c r="A527" s="21" t="inlineStr">
+        <is>
+          <t>slot09</t>
+        </is>
       </c>
       <c r="B527" s="21" t="inlineStr">
         <is>
-          <t>Mobilya Görünüm</t>
+          <t>null</t>
         </is>
       </c>
       <c r="C527" s="21" t="inlineStr">
         <is>
-          <t>furnView</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D527" s="21" t="inlineStr">
         <is>
-          <t>FURNITURE_VIEW</t>
+          <t>null</t>
         </is>
       </c>
       <c r="E527" s="21" t="inlineStr">
         <is>
-          <t>toggle-3-view</t>
+          <t>null</t>
         </is>
       </c>
       <c r="F527" s="21" t="n"/>
@@ -29262,11 +29266,10 @@
       <c r="N606" s="20" t="n"/>
       <c r="O606" s="20" t="n"/>
     </row>
-    <row r="607"/>
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>▌ SAHNE 5  —  Mobilya Editörü  ·  İç Mekan Dekorasyon</t>
+          <t>▌ SAHNE 4  —  Mobilya Editörü  ·  İç Mekan Dekorasyon</t>
         </is>
       </c>
     </row>

</xml_diff>